<commit_message>
ya pokoknya semuanya lah (buat di deploy)
</commit_message>
<xml_diff>
--- a/ExcelImport.xlsx
+++ b/ExcelImport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Codingan Kuliah\PADB\UCP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DBFF1B3-2812-4160-9F6A-C246EEF3F92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D4B799-75B0-403D-AF32-573690903AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0637EDC6-8E02-4033-B229-65E54DA3B240}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>NIM</t>
   </si>
@@ -48,6 +48,12 @@
   </si>
   <si>
     <t>Jurusan</t>
+  </si>
+  <si>
+    <t>Muhammad Fajri</t>
+  </si>
+  <si>
+    <t>Sistem Informasi</t>
   </si>
 </sst>
 </file>
@@ -419,8 +425,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0249797E-4A88-4017-B181-4F76C8684D99}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="15.21875" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -431,6 +441,17 @@
       </c>
       <c r="C1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>20240006</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>